<commit_message>
Update DCF model notes
</commit_message>
<xml_diff>
--- a/data/Stantec_DCF_Model.xlsx
+++ b/data/Stantec_DCF_Model.xlsx
@@ -33,88 +33,88 @@
     <t xml:space="preserve">Stantec Inc. (TSX/NYSE: STN) — Forecast &amp; DCF Model</t>
   </si>
   <si>
-    <t xml:space="preserve">C$ millions unless stated. Built to follow the Stantec Build Guide, step by step.</t>
+    <t xml:space="preserve">C$ millions unless stated. Five-year forecast and DCF valuation of Stantec built from its public filings. Prepared by Muhammad Ahsan, October 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Legend</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue = number typed in (from a report, or your assumption)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Black = formula (don't type over it)</t>
+    <t xml:space="preserve">Blue = hard-coded input (from a filing, or an assumption)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Black = formula</t>
   </si>
   <si>
     <t xml:space="preserve">Green = link pulled from another tab</t>
   </si>
   <si>
-    <t xml:space="preserve">Yellow = you fill this in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How to type numbers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example: gross revenue of $8,144.2 million is typed as 8144.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Percentages: type 24% (Excel stores it as 0.24)</t>
+    <t xml:space="preserve">Yellow = market inputs as of October 2026 (risk-free rate, beta, share price)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conventions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amounts in C$ millions (gross revenue of $8,144.2 million is shown as 8,144.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percentages are stored as decimals (24% = 0.24)</t>
   </si>
   <si>
     <t xml:space="preserve">Costs</t>
   </si>
   <si>
-    <t xml:space="preserve">Type costs and cash outflows (capex, dividends) as positive numbers; formulas subtract them</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Order of work</t>
+    <t xml:space="preserve">Costs and cash outflows (capex, dividends) are entered as positive numbers; formulas subtract them</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model structure</t>
   </si>
   <si>
     <t xml:space="preserve">1. Historicals</t>
   </si>
   <si>
-    <t xml:space="preserve">FY2024–25 income statement is already entered from the results release. Fill the yellow cells: the FY2023 column, plus the balance sheet and cash flow. FY2025 balance sheet is required; the rest is for ratios. The Check row must read 0.</t>
+    <t xml:space="preserve">FY2023–2025 income statement, balance sheet and cash flow from Stantec's results release and annual reports. The check row ties calculated net income to the reported figure.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Ratios</t>
   </si>
   <si>
-    <t xml:space="preserve">Automatic. Compare FY2025 with the build guide.</t>
+    <t xml:space="preserve">Growth, margins, cash conversion, leverage, DSO, working capital and return on equity, calculated from the historicals.</t>
   </si>
   <si>
     <t xml:space="preserve">3. Assumptions</t>
   </si>
   <si>
-    <t xml:space="preserve">Review the base case. Fill the 3 yellow market inputs: 10-year Government of Canada yield, beta (Yahoo Finance, STN.TO), today's share price.</t>
+    <t xml:space="preserve">Base-case forecast drivers anchored to management guidance, plus valuation and market inputs (Government of Canada 10-year yield, beta, share price).</t>
   </si>
   <si>
     <t xml:space="preserve">4. Forecast</t>
   </si>
   <si>
-    <t xml:space="preserve">Automatic. FY2026 should match the guide's check column.</t>
+    <t xml:space="preserve">FY2026–2030 forecast from net revenue down to unlevered free cash flow, driven by the Assumptions tab.</t>
   </si>
   <si>
     <t xml:space="preserve">5. WACC</t>
   </si>
   <si>
-    <t xml:space="preserve">Automatic once market inputs are in. Expect roughly 8–9.5%.</t>
+    <t xml:space="preserve">Cost of equity (CAPM), after-tax cost of debt and market-value capital weights.</t>
   </si>
   <si>
     <t xml:space="preserve">6. DCF</t>
   </si>
   <si>
-    <t xml:space="preserve">Automatic, including the sensitivity table (build guide Step 7 is already done).</t>
+    <t xml:space="preserve">Discounts FY2026–2030 free cash flow and a Gordon-growth terminal value to Dec 31, 2025, bridges enterprise value to value per share, and runs a WACC × terminal growth sensitivity table.</t>
   </si>
   <si>
     <t xml:space="preserve">7. Comps</t>
   </si>
   <si>
-    <t xml:space="preserve">Fill EV/EBITDA for the four peers and Stantec, and Stantec's EBITDA, all from the same source.</t>
+    <t xml:space="preserve">EV/EBITDA for four engineering and design peers (WSP, AECOM, Tetra Tech, Jacobs) from a single source; the peer median is applied to Stantec's EBITDA.</t>
   </si>
   <si>
     <t xml:space="preserve">8. Summary</t>
   </si>
   <si>
-    <t xml:space="preserve">Add your name and date, check the verdict, and edit the bullets in your own words. Export this tab to PDF.</t>
+    <t xml:space="preserve">One-page valuation summary: DCF and comps value per share vs. the share price, key assumptions, upside drivers and risks.</t>
   </si>
   <si>
     <t xml:space="preserve">Sources</t>
@@ -156,7 +156,7 @@
     <t xml:space="preserve">Subconsultant and other direct expenses</t>
   </si>
   <si>
-    <t xml:space="preserve">FY2024–25 derived as gross − net revenue from the release; confirm against the annual report line.</t>
+    <t xml:space="preserve">FY2024–25 derived as gross revenue less net revenue from the results release.</t>
   </si>
   <si>
     <t xml:space="preserve">Net revenue</t>
@@ -207,13 +207,13 @@
     <t xml:space="preserve">Reported net income</t>
   </si>
   <si>
-    <t xml:space="preserve">Type the net income shown in the report</t>
+    <t xml:space="preserve">Net income as reported</t>
   </si>
   <si>
     <t xml:space="preserve">Check (must be 0)</t>
   </si>
   <si>
-    <t xml:space="preserve">Not 0 = a mistyped number or a missing line</t>
+    <t xml:space="preserve">Calculated less reported net income</t>
   </si>
   <si>
     <t xml:space="preserve">Balance sheet (Dec 31)</t>
@@ -222,19 +222,19 @@
     <t xml:space="preserve">Cash and cash equivalents</t>
   </si>
   <si>
-    <t xml:space="preserve">FY2025 required (used in net debt and the DCF)</t>
+    <t xml:space="preserve">Used in net debt and the DCF</t>
   </si>
   <si>
     <t xml:space="preserve">Trade and other receivables</t>
   </si>
   <si>
-    <t xml:space="preserve">FY2025 required (drives working capital %)</t>
+    <t xml:space="preserve">Drives the working capital assumption</t>
   </si>
   <si>
     <t xml:space="preserve">Contract assets (work done, not yet billed)</t>
   </si>
   <si>
-    <t xml:space="preserve">FY2025 required</t>
+    <t xml:space="preserve">Used in working capital</t>
   </si>
   <si>
     <t xml:space="preserve">Trade and other payables</t>
@@ -246,7 +246,7 @@
     <t xml:space="preserve">Total debt (excl. lease liabilities)</t>
   </si>
   <si>
-    <t xml:space="preserve">FY2024–25: "Total long-term debt" from the results release. Confirm it includes the current portion and excludes leases.</t>
+    <t xml:space="preserve">FY2024–25: total long-term debt from the results release, including the current portion and excluding lease liabilities.</t>
   </si>
   <si>
     <t xml:space="preserve">Total shareholders' equity</t>
@@ -264,7 +264,7 @@
     <t xml:space="preserve">Capex (property &amp; equipment + intangibles)</t>
   </si>
   <si>
-    <t xml:space="preserve">Type as a positive number</t>
+    <t xml:space="preserve">Entered as a positive number</t>
   </si>
   <si>
     <t xml:space="preserve">Business acquisitions</t>
@@ -276,7 +276,7 @@
     <t xml:space="preserve">Key Ratios</t>
   </si>
   <si>
-    <t xml:space="preserve">All automatic. FY2025 should match the build guide.</t>
+    <t xml:space="preserve">Calculated from the Historicals tab.</t>
   </si>
   <si>
     <t xml:space="preserve">Ratio</t>
@@ -453,7 +453,7 @@
     <t xml:space="preserve">Midpoint of management's 1.4–1.8% guidance.</t>
   </si>
   <si>
-    <t xml:space="preserve">From your FY2025 balance sheet (Ratios tab); held flat. Shows "-" until the balance sheet is filled in.</t>
+    <t xml:space="preserve">FY2025 level from the Ratios tab, held flat.</t>
   </si>
   <si>
     <t xml:space="preserve">Valuation inputs</t>
@@ -462,25 +462,25 @@
     <t xml:space="preserve">Value</t>
   </si>
   <si>
-    <t xml:space="preserve">Why / where to find it</t>
+    <t xml:space="preserve">Rationale / source</t>
   </si>
   <si>
     <t xml:space="preserve">Terminal growth (g)</t>
   </si>
   <si>
-    <t xml:space="preserve">Long-run growth after 2030: roughly inflation plus a little. Must stay below WACC.</t>
+    <t xml:space="preserve">Long-run growth after 2030, roughly inflation plus modest real growth; must stay below WACC.</t>
   </si>
   <si>
     <t xml:space="preserve">Equity risk premium</t>
   </si>
   <si>
-    <t xml:space="preserve">Extra return investors demand for stocks over bonds; a common assumption.</t>
+    <t xml:space="preserve">Equity risk premium over government bonds; a standard assumption.</t>
   </si>
   <si>
     <t xml:space="preserve">Pre-tax cost of debt</t>
   </si>
   <si>
-    <t xml:space="preserve">Placeholder. Replace with the average rate on Stantec's notes (debt note in the annual report) if you find it.</t>
+    <t xml:space="preserve">Assumed pre-tax cost of Stantec's borrowings; debt is about 14% of capital, so WACC is not very sensitive to it.</t>
   </si>
   <si>
     <t xml:space="preserve">Diluted shares (millions)</t>
@@ -489,16 +489,16 @@
     <t xml:space="preserve">Weighted average diluted shares: 114,066,995 (results release, Feb 25, 2026).</t>
   </si>
   <si>
-    <t xml:space="preserve">Market inputs — fill in today's values</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Where to find it</t>
+    <t xml:space="preserve">Market inputs (October 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source</t>
   </si>
   <si>
     <t xml:space="preserve">Risk-free rate</t>
   </si>
   <si>
-    <t xml:space="preserve">Government of Canada 10-year bond yield (Bank of Canada website). Type as %, e.g. 3.2%.</t>
+    <t xml:space="preserve">Government of Canada 10-year bond yield (Bank of Canada).</t>
   </si>
   <si>
     <t xml:space="preserve">Beta</t>
@@ -585,7 +585,7 @@
     <t xml:space="preserve">Cost of equity</t>
   </si>
   <si>
-    <t xml:space="preserve">CAPM: safe return + beta × extra return for risk</t>
+    <t xml:space="preserve">CAPM: risk-free rate + beta × equity risk premium</t>
   </si>
   <si>
     <t xml:space="preserve">Tax rate</t>
@@ -624,7 +624,7 @@
     <t xml:space="preserve">WACC</t>
   </si>
   <si>
-    <t xml:space="preserve">Shows "-" until the market inputs are filled in</t>
+    <t xml:space="preserve">Discount rate used in the DCF</t>
   </si>
   <si>
     <t xml:space="preserve">DCF Valuation</t>
@@ -666,7 +666,7 @@
     <t xml:space="preserve">PV of terminal value</t>
   </si>
   <si>
-    <t xml:space="preserve">shrunk back five years</t>
+    <t xml:space="preserve">discounted back five years</t>
   </si>
   <si>
     <t xml:space="preserve">Enterprise value</t>
@@ -702,13 +702,13 @@
     <t xml:space="preserve">WACC ↓  g →</t>
   </si>
   <si>
-    <t xml:space="preserve">Each cell reruns the full DCF at that WACC and growth rate. Find the cell closest to your WACC and 2.5% for your base case.</t>
+    <t xml:space="preserve">Each cell reruns the full DCF at that WACC and terminal growth rate. Base case: 7.3% WACC and 2.5% growth gives $138.00.</t>
   </si>
   <si>
     <t xml:space="preserve">Peer Comparison (EV/EBITDA)</t>
   </si>
   <si>
-    <t xml:space="preserve">Take every multiple, and Stantec's EBITDA, from ONE source (Yahoo Finance Statistics tab or stockanalysis.com) so definitions match.</t>
+    <t xml:space="preserve">All multiples and Stantec's EBITDA come from one data source so definitions match.</t>
   </si>
   <si>
     <t xml:space="preserve">Company</t>

</xml_diff>